<commit_message>
Updates to BOM and placements.
</commit_message>
<xml_diff>
--- a/PCBs/expansion-stepper1/MakerPnPControl-stepper1_variant1_cpl.xlsx
+++ b/PCBs/expansion-stepper1/MakerPnPControl-stepper1_variant1_cpl.xlsx
@@ -1,27 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Hydra\Documents\DipTrace\Projects\MakerPnPControl\PCBs\expansion-stepper1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{51E30F9F-67BB-4A02-ACF7-C7EB37E4B5FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{469F2C91-DF2A-41F7-A28E-179EA18FA9FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="26670" yWindow="17040" windowWidth="25155" windowHeight="9495" xr2:uid="{2576EC9E-D0E2-4B69-A6A4-5FEBE97C57C4}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="25155" windowHeight="9495" xr2:uid="{2576EC9E-D0E2-4B69-A6A4-5FEBE97C57C4}"/>
   </bookViews>
   <sheets>
     <sheet name="MakerPnPControl-stepper1_varian" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="685" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="709" uniqueCount="248">
   <si>
     <t>RefDes</t>
   </si>
@@ -732,6 +745,39 @@
   </si>
   <si>
     <t>Layer</t>
+  </si>
+  <si>
+    <t>R65</t>
+  </si>
+  <si>
+    <t>RC2512JK-073K3L</t>
+  </si>
+  <si>
+    <t>RV1</t>
+  </si>
+  <si>
+    <t>BOURNS</t>
+  </si>
+  <si>
+    <t>AV20K1210401NIR1</t>
+  </si>
+  <si>
+    <t>RV2</t>
+  </si>
+  <si>
+    <t>RV3</t>
+  </si>
+  <si>
+    <t>RV4</t>
+  </si>
+  <si>
+    <t>X2</t>
+  </si>
+  <si>
+    <t>XFCN</t>
+  </si>
+  <si>
+    <t>XF-154</t>
   </si>
 </sst>
 </file>
@@ -1592,7 +1638,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08333570-5FD6-4524-979B-E57B0629D686}">
-  <dimension ref="A1:E169"/>
+  <dimension ref="A1:E175"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -1887,7 +1933,7 @@
       </c>
       <c r="C14">
         <f>Sheet1!G14</f>
-        <v>162.15</v>
+        <v>160.9</v>
       </c>
       <c r="D14" t="str">
         <f>Sheet1!E14</f>
@@ -1895,7 +1941,7 @@
       </c>
       <c r="E14">
         <f>ROUND(Sheet1!H14,0)</f>
-        <v>90</v>
+        <v>180</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -2345,7 +2391,7 @@
       </c>
       <c r="B35">
         <f>Sheet1!F35</f>
-        <v>37.75</v>
+        <v>37.875</v>
       </c>
       <c r="C35">
         <f>Sheet1!G35</f>
@@ -2367,7 +2413,7 @@
       </c>
       <c r="B36">
         <f>Sheet1!F36</f>
-        <v>41.75</v>
+        <v>42.125</v>
       </c>
       <c r="C36">
         <f>Sheet1!G36</f>
@@ -2521,7 +2567,7 @@
       </c>
       <c r="B43">
         <f>Sheet1!F43</f>
-        <v>28.25</v>
+        <v>27.875</v>
       </c>
       <c r="C43">
         <f>Sheet1!G43</f>
@@ -2543,7 +2589,7 @@
       </c>
       <c r="B44">
         <f>Sheet1!F44</f>
-        <v>32.25</v>
+        <v>32.125</v>
       </c>
       <c r="C44">
         <f>Sheet1!G44</f>
@@ -3159,11 +3205,11 @@
       </c>
       <c r="B72">
         <f>Sheet1!F72</f>
-        <v>23</v>
+        <v>45.5</v>
       </c>
       <c r="C72">
         <f>Sheet1!G72</f>
-        <v>161.9</v>
+        <v>164.52500000000001</v>
       </c>
       <c r="D72" t="str">
         <f>Sheet1!E72</f>
@@ -3185,7 +3231,7 @@
       </c>
       <c r="C73">
         <f>Sheet1!G73</f>
-        <v>149.69999999999999</v>
+        <v>149.44999999999999</v>
       </c>
       <c r="D73" t="str">
         <f>Sheet1!E73</f>
@@ -3251,7 +3297,7 @@
       </c>
       <c r="C76">
         <f>Sheet1!G76</f>
-        <v>43.1</v>
+        <v>43.35</v>
       </c>
       <c r="D76" t="str">
         <f>Sheet1!E76</f>
@@ -3273,7 +3319,7 @@
       </c>
       <c r="C77">
         <f>Sheet1!G77</f>
-        <v>169.875</v>
+        <v>170.125</v>
       </c>
       <c r="D77" t="str">
         <f>Sheet1!E77</f>
@@ -3295,7 +3341,7 @@
       </c>
       <c r="C78">
         <f>Sheet1!G78</f>
-        <v>168.4</v>
+        <v>168.77500000000001</v>
       </c>
       <c r="D78" t="str">
         <f>Sheet1!E78</f>
@@ -4457,11 +4503,11 @@
       </c>
       <c r="B131">
         <f>Sheet1!F131</f>
-        <v>48.75</v>
+        <v>51.5</v>
       </c>
       <c r="C131">
         <f>Sheet1!G131</f>
-        <v>164.21199999999999</v>
+        <v>163.77500000000001</v>
       </c>
       <c r="D131" t="str">
         <f>Sheet1!E131</f>
@@ -4479,11 +4525,11 @@
       </c>
       <c r="B132">
         <f>Sheet1!F132</f>
-        <v>48.75</v>
+        <v>50</v>
       </c>
       <c r="C132">
         <f>Sheet1!G132</f>
-        <v>163.21199999999999</v>
+        <v>164.27500000000001</v>
       </c>
       <c r="D132" t="str">
         <f>Sheet1!E132</f>
@@ -4491,7 +4537,7 @@
       </c>
       <c r="E132">
         <f>ROUND(Sheet1!H132,0)</f>
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.25">
@@ -5069,15 +5115,15 @@
     <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" t="str">
         <f>Sheet1!A159</f>
-        <v>R155</v>
+        <v>R65</v>
       </c>
       <c r="B159">
         <f>Sheet1!F159</f>
-        <v>24.45</v>
+        <v>46.125</v>
       </c>
       <c r="C159">
         <f>Sheet1!G159</f>
-        <v>96.4</v>
+        <v>156.27500000000001</v>
       </c>
       <c r="D159" t="str">
         <f>Sheet1!E159</f>
@@ -5085,17 +5131,17 @@
       </c>
       <c r="E159">
         <f>ROUND(Sheet1!H159,0)</f>
-        <v>90</v>
+        <v>0</v>
       </c>
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" t="str">
         <f>Sheet1!A160</f>
-        <v>R156</v>
+        <v>R155</v>
       </c>
       <c r="B160">
         <f>Sheet1!F160</f>
-        <v>45.55</v>
+        <v>24.45</v>
       </c>
       <c r="C160">
         <f>Sheet1!G160</f>
@@ -5107,21 +5153,21 @@
       </c>
       <c r="E160">
         <f>ROUND(Sheet1!H160,0)</f>
-        <v>-90</v>
+        <v>90</v>
       </c>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" t="str">
         <f>Sheet1!A161</f>
-        <v>U1</v>
+        <v>R156</v>
       </c>
       <c r="B161">
         <f>Sheet1!F161</f>
-        <v>20.75</v>
+        <v>45.55</v>
       </c>
       <c r="C161">
         <f>Sheet1!G161</f>
-        <v>157.65</v>
+        <v>96.4</v>
       </c>
       <c r="D161" t="str">
         <f>Sheet1!E161</f>
@@ -5129,21 +5175,21 @@
       </c>
       <c r="E161">
         <f>ROUND(Sheet1!H161,0)</f>
-        <v>0</v>
+        <v>-90</v>
       </c>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" t="str">
         <f>Sheet1!A162</f>
-        <v>U2</v>
+        <v>RV1</v>
       </c>
       <c r="B162">
         <f>Sheet1!F162</f>
-        <v>35</v>
+        <v>25.312999999999999</v>
       </c>
       <c r="C162">
         <f>Sheet1!G162</f>
-        <v>86.9</v>
+        <v>43.024999999999999</v>
       </c>
       <c r="D162" t="str">
         <f>Sheet1!E162</f>
@@ -5151,21 +5197,21 @@
       </c>
       <c r="E162">
         <f>ROUND(Sheet1!H162,0)</f>
-        <v>180</v>
+        <v>90</v>
       </c>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" t="str">
         <f>Sheet1!A163</f>
-        <v>U3</v>
+        <v>RV2</v>
       </c>
       <c r="B163">
         <f>Sheet1!F163</f>
-        <v>49.25</v>
+        <v>44.688000000000002</v>
       </c>
       <c r="C163">
         <f>Sheet1!G163</f>
-        <v>160.65</v>
+        <v>43.024999999999999</v>
       </c>
       <c r="D163" t="str">
         <f>Sheet1!E163</f>
@@ -5173,21 +5219,21 @@
       </c>
       <c r="E163">
         <f>ROUND(Sheet1!H163,0)</f>
-        <v>180</v>
+        <v>-90</v>
       </c>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" t="str">
         <f>Sheet1!A164</f>
-        <v>U4</v>
+        <v>RV3</v>
       </c>
       <c r="B164">
         <f>Sheet1!F164</f>
-        <v>18</v>
+        <v>44.688000000000002</v>
       </c>
       <c r="C164">
         <f>Sheet1!G164</f>
-        <v>32.15</v>
+        <v>149.77500000000001</v>
       </c>
       <c r="D164" t="str">
         <f>Sheet1!E164</f>
@@ -5195,21 +5241,21 @@
       </c>
       <c r="E164">
         <f>ROUND(Sheet1!H164,0)</f>
-        <v>0</v>
+        <v>-90</v>
       </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" t="str">
         <f>Sheet1!A165</f>
-        <v>U5</v>
+        <v>RV4</v>
       </c>
       <c r="B165">
         <f>Sheet1!F165</f>
-        <v>35</v>
+        <v>25.312999999999999</v>
       </c>
       <c r="C165">
         <f>Sheet1!G165</f>
-        <v>32.15</v>
+        <v>149.77500000000001</v>
       </c>
       <c r="D165" t="str">
         <f>Sheet1!E165</f>
@@ -5217,21 +5263,21 @@
       </c>
       <c r="E165">
         <f>ROUND(Sheet1!H165,0)</f>
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" t="str">
         <f>Sheet1!A166</f>
-        <v>U6</v>
+        <v>U1</v>
       </c>
       <c r="B166">
         <f>Sheet1!F166</f>
-        <v>35</v>
+        <v>20.75</v>
       </c>
       <c r="C166">
         <f>Sheet1!G166</f>
-        <v>105.9</v>
+        <v>157.65</v>
       </c>
       <c r="D166" t="str">
         <f>Sheet1!E166</f>
@@ -5245,15 +5291,15 @@
     <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" t="str">
         <f>Sheet1!A167</f>
-        <v>U7</v>
+        <v>U2</v>
       </c>
       <c r="B167">
         <f>Sheet1!F167</f>
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="C167">
         <f>Sheet1!G167</f>
-        <v>32.15</v>
+        <v>86.9</v>
       </c>
       <c r="D167" t="str">
         <f>Sheet1!E167</f>
@@ -5261,21 +5307,21 @@
       </c>
       <c r="E167">
         <f>ROUND(Sheet1!H167,0)</f>
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" t="str">
         <f>Sheet1!A168</f>
-        <v>U42</v>
+        <v>U3</v>
       </c>
       <c r="B168">
         <f>Sheet1!F168</f>
-        <v>19.899999999999999</v>
+        <v>49.25</v>
       </c>
       <c r="C168">
         <f>Sheet1!G168</f>
-        <v>96.4</v>
+        <v>160.65</v>
       </c>
       <c r="D168" t="str">
         <f>Sheet1!E168</f>
@@ -5283,21 +5329,21 @@
       </c>
       <c r="E168">
         <f>ROUND(Sheet1!H168,0)</f>
-        <v>-180</v>
+        <v>180</v>
       </c>
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" t="str">
         <f>Sheet1!A169</f>
-        <v>U43</v>
+        <v>U4</v>
       </c>
       <c r="B169">
         <f>Sheet1!F169</f>
-        <v>50.1</v>
+        <v>18</v>
       </c>
       <c r="C169">
         <f>Sheet1!G169</f>
-        <v>96.4</v>
+        <v>32.15</v>
       </c>
       <c r="D169" t="str">
         <f>Sheet1!E169</f>
@@ -5305,6 +5351,138 @@
       </c>
       <c r="E169">
         <f>ROUND(Sheet1!H169,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A170" t="str">
+        <f>Sheet1!A170</f>
+        <v>U5</v>
+      </c>
+      <c r="B170">
+        <f>Sheet1!F170</f>
+        <v>35</v>
+      </c>
+      <c r="C170">
+        <f>Sheet1!G170</f>
+        <v>32.15</v>
+      </c>
+      <c r="D170" t="str">
+        <f>Sheet1!E170</f>
+        <v>Top</v>
+      </c>
+      <c r="E170">
+        <f>ROUND(Sheet1!H170,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A171" t="str">
+        <f>Sheet1!A171</f>
+        <v>U6</v>
+      </c>
+      <c r="B171">
+        <f>Sheet1!F171</f>
+        <v>35</v>
+      </c>
+      <c r="C171">
+        <f>Sheet1!G171</f>
+        <v>105.9</v>
+      </c>
+      <c r="D171" t="str">
+        <f>Sheet1!E171</f>
+        <v>Top</v>
+      </c>
+      <c r="E171">
+        <f>ROUND(Sheet1!H171,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A172" t="str">
+        <f>Sheet1!A172</f>
+        <v>U7</v>
+      </c>
+      <c r="B172">
+        <f>Sheet1!F172</f>
+        <v>52</v>
+      </c>
+      <c r="C172">
+        <f>Sheet1!G172</f>
+        <v>32.15</v>
+      </c>
+      <c r="D172" t="str">
+        <f>Sheet1!E172</f>
+        <v>Top</v>
+      </c>
+      <c r="E172">
+        <f>ROUND(Sheet1!H172,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A173" t="str">
+        <f>Sheet1!A173</f>
+        <v>U42</v>
+      </c>
+      <c r="B173">
+        <f>Sheet1!F173</f>
+        <v>19.899999999999999</v>
+      </c>
+      <c r="C173">
+        <f>Sheet1!G173</f>
+        <v>96.4</v>
+      </c>
+      <c r="D173" t="str">
+        <f>Sheet1!E173</f>
+        <v>Top</v>
+      </c>
+      <c r="E173">
+        <f>ROUND(Sheet1!H173,0)</f>
+        <v>-180</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A174" t="str">
+        <f>Sheet1!A174</f>
+        <v>U43</v>
+      </c>
+      <c r="B174">
+        <f>Sheet1!F174</f>
+        <v>50.1</v>
+      </c>
+      <c r="C174">
+        <f>Sheet1!G174</f>
+        <v>96.4</v>
+      </c>
+      <c r="D174" t="str">
+        <f>Sheet1!E174</f>
+        <v>Top</v>
+      </c>
+      <c r="E174">
+        <f>ROUND(Sheet1!H174,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A175" t="str">
+        <f>Sheet1!A175</f>
+        <v>X2</v>
+      </c>
+      <c r="B175">
+        <f>Sheet1!F175</f>
+        <v>35</v>
+      </c>
+      <c r="C175">
+        <f>Sheet1!G175</f>
+        <v>170.52500000000001</v>
+      </c>
+      <c r="D175" t="str">
+        <f>Sheet1!E175</f>
+        <v>Top</v>
+      </c>
+      <c r="E175">
+        <f>ROUND(Sheet1!H175,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -5315,7 +5493,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2F4F7E3-3481-49B5-9745-DA9C3836DC43}">
-  <dimension ref="A1:H169"/>
+  <dimension ref="A1:H175"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5676,10 +5854,10 @@
         <v>35</v>
       </c>
       <c r="G14">
-        <v>162.15</v>
+        <v>160.9</v>
       </c>
       <c r="H14">
-        <v>90</v>
+        <v>180</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
@@ -6219,7 +6397,7 @@
         <v>11</v>
       </c>
       <c r="F35">
-        <v>37.75</v>
+        <v>37.875</v>
       </c>
       <c r="G35">
         <v>144.15</v>
@@ -6245,7 +6423,7 @@
         <v>11</v>
       </c>
       <c r="F36">
-        <v>41.75</v>
+        <v>42.125</v>
       </c>
       <c r="G36">
         <v>144.15</v>
@@ -6427,7 +6605,7 @@
         <v>11</v>
       </c>
       <c r="F43">
-        <v>28.25</v>
+        <v>27.875</v>
       </c>
       <c r="G43">
         <v>144.15</v>
@@ -6453,7 +6631,7 @@
         <v>11</v>
       </c>
       <c r="F44">
-        <v>32.25</v>
+        <v>32.125</v>
       </c>
       <c r="G44">
         <v>144.15</v>
@@ -7181,10 +7359,10 @@
         <v>11</v>
       </c>
       <c r="F72">
-        <v>23</v>
+        <v>45.5</v>
       </c>
       <c r="G72">
-        <v>161.9</v>
+        <v>164.52500000000001</v>
       </c>
       <c r="H72">
         <v>0</v>
@@ -7210,7 +7388,7 @@
         <v>35</v>
       </c>
       <c r="G73">
-        <v>149.69999999999999</v>
+        <v>149.44999999999999</v>
       </c>
       <c r="H73">
         <v>180</v>
@@ -7288,7 +7466,7 @@
         <v>35</v>
       </c>
       <c r="G76">
-        <v>43.1</v>
+        <v>43.35</v>
       </c>
       <c r="H76">
         <v>0</v>
@@ -7314,7 +7492,7 @@
         <v>46.95</v>
       </c>
       <c r="G77">
-        <v>169.875</v>
+        <v>170.125</v>
       </c>
       <c r="H77">
         <v>0</v>
@@ -7340,7 +7518,7 @@
         <v>23</v>
       </c>
       <c r="G78">
-        <v>168.4</v>
+        <v>168.77500000000001</v>
       </c>
       <c r="H78">
         <v>180</v>
@@ -8715,10 +8893,10 @@
         <v>11</v>
       </c>
       <c r="F131">
-        <v>48.75</v>
+        <v>51.5</v>
       </c>
       <c r="G131">
-        <v>164.21199999999999</v>
+        <v>163.77500000000001</v>
       </c>
       <c r="H131">
         <v>0</v>
@@ -8741,13 +8919,13 @@
         <v>11</v>
       </c>
       <c r="F132">
-        <v>48.75</v>
+        <v>50</v>
       </c>
       <c r="G132">
-        <v>163.21199999999999</v>
+        <v>164.27500000000001</v>
       </c>
       <c r="H132">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="133" spans="1:8" x14ac:dyDescent="0.25">
@@ -9428,13 +9606,13 @@
     </row>
     <row r="159" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>215</v>
+        <v>237</v>
       </c>
       <c r="B159" t="s">
         <v>16</v>
       </c>
       <c r="C159" t="s">
-        <v>216</v>
+        <v>238</v>
       </c>
       <c r="D159" t="b">
         <v>1</v>
@@ -9443,18 +9621,18 @@
         <v>11</v>
       </c>
       <c r="F159">
-        <v>24.45</v>
+        <v>46.125</v>
       </c>
       <c r="G159">
-        <v>96.4</v>
+        <v>156.27500000000001</v>
       </c>
       <c r="H159">
-        <v>90</v>
+        <v>0</v>
       </c>
     </row>
     <row r="160" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B160" t="s">
         <v>16</v>
@@ -9469,24 +9647,24 @@
         <v>11</v>
       </c>
       <c r="F160">
-        <v>45.55</v>
+        <v>24.45</v>
       </c>
       <c r="G160">
         <v>96.4</v>
       </c>
       <c r="H160">
-        <v>-90</v>
+        <v>90</v>
       </c>
     </row>
     <row r="161" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B161" t="s">
-        <v>219</v>
+        <v>16</v>
       </c>
       <c r="C161" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="D161" t="b">
         <v>1</v>
@@ -9495,24 +9673,24 @@
         <v>11</v>
       </c>
       <c r="F161">
-        <v>20.75</v>
+        <v>45.55</v>
       </c>
       <c r="G161">
-        <v>157.65</v>
+        <v>96.4</v>
       </c>
       <c r="H161">
-        <v>0</v>
+        <v>-90</v>
       </c>
     </row>
     <row r="162" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>221</v>
+        <v>239</v>
       </c>
       <c r="B162" t="s">
-        <v>222</v>
+        <v>240</v>
       </c>
       <c r="C162" t="s">
-        <v>223</v>
+        <v>241</v>
       </c>
       <c r="D162" t="b">
         <v>1</v>
@@ -9521,24 +9699,24 @@
         <v>11</v>
       </c>
       <c r="F162">
-        <v>35</v>
+        <v>25.312999999999999</v>
       </c>
       <c r="G162">
-        <v>86.9</v>
+        <v>43.024999999999999</v>
       </c>
       <c r="H162">
-        <v>180</v>
+        <v>90</v>
       </c>
     </row>
     <row r="163" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>224</v>
+        <v>242</v>
       </c>
       <c r="B163" t="s">
-        <v>219</v>
+        <v>240</v>
       </c>
       <c r="C163" t="s">
-        <v>220</v>
+        <v>241</v>
       </c>
       <c r="D163" t="b">
         <v>1</v>
@@ -9547,24 +9725,24 @@
         <v>11</v>
       </c>
       <c r="F163">
-        <v>49.25</v>
+        <v>44.688000000000002</v>
       </c>
       <c r="G163">
-        <v>160.65</v>
+        <v>43.024999999999999</v>
       </c>
       <c r="H163">
-        <v>180</v>
+        <v>-90</v>
       </c>
     </row>
     <row r="164" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>225</v>
+        <v>243</v>
       </c>
       <c r="B164" t="s">
-        <v>219</v>
+        <v>240</v>
       </c>
       <c r="C164" t="s">
-        <v>226</v>
+        <v>241</v>
       </c>
       <c r="D164" t="b">
         <v>1</v>
@@ -9573,24 +9751,24 @@
         <v>11</v>
       </c>
       <c r="F164">
-        <v>18</v>
+        <v>44.688000000000002</v>
       </c>
       <c r="G164">
-        <v>32.15</v>
+        <v>149.77500000000001</v>
       </c>
       <c r="H164">
-        <v>0</v>
+        <v>-90</v>
       </c>
     </row>
     <row r="165" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>227</v>
+        <v>244</v>
       </c>
       <c r="B165" t="s">
-        <v>219</v>
+        <v>240</v>
       </c>
       <c r="C165" t="s">
-        <v>226</v>
+        <v>241</v>
       </c>
       <c r="D165" t="b">
         <v>1</v>
@@ -9599,24 +9777,24 @@
         <v>11</v>
       </c>
       <c r="F165">
-        <v>35</v>
+        <v>25.312999999999999</v>
       </c>
       <c r="G165">
-        <v>32.15</v>
+        <v>149.77500000000001</v>
       </c>
       <c r="H165">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="166" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>228</v>
+        <v>218</v>
       </c>
       <c r="B166" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="C166" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="D166" t="b">
         <v>1</v>
@@ -9625,10 +9803,10 @@
         <v>11</v>
       </c>
       <c r="F166">
-        <v>35</v>
+        <v>20.75</v>
       </c>
       <c r="G166">
-        <v>105.9</v>
+        <v>157.65</v>
       </c>
       <c r="H166">
         <v>0</v>
@@ -9636,13 +9814,13 @@
     </row>
     <row r="167" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="B167" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="C167" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D167" t="b">
         <v>1</v>
@@ -9651,24 +9829,24 @@
         <v>11</v>
       </c>
       <c r="F167">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="G167">
-        <v>32.15</v>
+        <v>86.9</v>
       </c>
       <c r="H167">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="168" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="B168" t="s">
         <v>219</v>
       </c>
       <c r="C168" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="D168" t="b">
         <v>1</v>
@@ -9677,38 +9855,194 @@
         <v>11</v>
       </c>
       <c r="F168">
-        <v>19.899999999999999</v>
+        <v>49.25</v>
       </c>
       <c r="G168">
-        <v>96.4</v>
+        <v>160.65</v>
       </c>
       <c r="H168">
-        <v>-179.99</v>
+        <v>180</v>
       </c>
     </row>
     <row r="169" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="B169" t="s">
         <v>219</v>
       </c>
       <c r="C169" t="s">
+        <v>226</v>
+      </c>
+      <c r="D169" t="b">
+        <v>1</v>
+      </c>
+      <c r="E169" t="s">
+        <v>11</v>
+      </c>
+      <c r="F169">
+        <v>18</v>
+      </c>
+      <c r="G169">
+        <v>32.15</v>
+      </c>
+      <c r="H169">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="170" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A170" t="s">
+        <v>227</v>
+      </c>
+      <c r="B170" t="s">
+        <v>219</v>
+      </c>
+      <c r="C170" t="s">
+        <v>226</v>
+      </c>
+      <c r="D170" t="b">
+        <v>1</v>
+      </c>
+      <c r="E170" t="s">
+        <v>11</v>
+      </c>
+      <c r="F170">
+        <v>35</v>
+      </c>
+      <c r="G170">
+        <v>32.15</v>
+      </c>
+      <c r="H170">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="171" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A171" t="s">
+        <v>228</v>
+      </c>
+      <c r="B171" t="s">
+        <v>222</v>
+      </c>
+      <c r="C171" t="s">
+        <v>223</v>
+      </c>
+      <c r="D171" t="b">
+        <v>1</v>
+      </c>
+      <c r="E171" t="s">
+        <v>11</v>
+      </c>
+      <c r="F171">
+        <v>35</v>
+      </c>
+      <c r="G171">
+        <v>105.9</v>
+      </c>
+      <c r="H171">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="172" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A172" t="s">
+        <v>229</v>
+      </c>
+      <c r="B172" t="s">
+        <v>219</v>
+      </c>
+      <c r="C172" t="s">
+        <v>226</v>
+      </c>
+      <c r="D172" t="b">
+        <v>1</v>
+      </c>
+      <c r="E172" t="s">
+        <v>11</v>
+      </c>
+      <c r="F172">
+        <v>52</v>
+      </c>
+      <c r="G172">
+        <v>32.15</v>
+      </c>
+      <c r="H172">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="173" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A173" t="s">
+        <v>230</v>
+      </c>
+      <c r="B173" t="s">
+        <v>219</v>
+      </c>
+      <c r="C173" t="s">
         <v>231</v>
       </c>
-      <c r="D169" t="b">
-        <v>1</v>
-      </c>
-      <c r="E169" t="s">
-        <v>11</v>
-      </c>
-      <c r="F169">
+      <c r="D173" t="b">
+        <v>1</v>
+      </c>
+      <c r="E173" t="s">
+        <v>11</v>
+      </c>
+      <c r="F173">
+        <v>19.899999999999999</v>
+      </c>
+      <c r="G173">
+        <v>96.4</v>
+      </c>
+      <c r="H173">
+        <v>-179.99</v>
+      </c>
+    </row>
+    <row r="174" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A174" t="s">
+        <v>232</v>
+      </c>
+      <c r="B174" t="s">
+        <v>219</v>
+      </c>
+      <c r="C174" t="s">
+        <v>231</v>
+      </c>
+      <c r="D174" t="b">
+        <v>1</v>
+      </c>
+      <c r="E174" t="s">
+        <v>11</v>
+      </c>
+      <c r="F174">
         <v>50.1</v>
       </c>
-      <c r="G169">
+      <c r="G174">
         <v>96.4</v>
       </c>
-      <c r="H169">
+      <c r="H174">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="175" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A175" t="s">
+        <v>245</v>
+      </c>
+      <c r="B175" t="s">
+        <v>246</v>
+      </c>
+      <c r="C175" t="s">
+        <v>247</v>
+      </c>
+      <c r="D175" t="b">
+        <v>1</v>
+      </c>
+      <c r="E175" t="s">
+        <v>11</v>
+      </c>
+      <c r="F175">
+        <v>35</v>
+      </c>
+      <c r="G175">
+        <v>170.52500000000001</v>
+      </c>
+      <c r="H175">
         <v>0</v>
       </c>
     </row>

</xml_diff>